<commit_message>
Agrega mapas LATAM al estudio de mercado (ES/EN) y hoja Mapas al plan de marketing
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012axCVDM5kAgj1VFnxhpsuM
</commit_message>
<xml_diff>
--- a/propuesta-clt/Plan_Marketing_CLT_Mexico_Latam.xlsx
+++ b/propuesta-clt/Plan_Marketing_CLT_Mexico_Latam.xlsx
@@ -26,6 +26,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latinoamérica" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedir a CLT" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riesgos" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapas" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -271,6 +272,61 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="8143875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>49</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="8143875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4653,6 +4709,51 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001B1F3B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:A49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Mapas de prospectos LATAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Estrella dorada: cuenta 80/20 en México o prioridad A en el resto de LATAM. Ubicación aproximada por ciudad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>OEM — maquila de exportación</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Estampadores y fabricantes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>